<commit_message>
Keeping MMUser up to date
</commit_message>
<xml_diff>
--- a/config/acquisitionConfig/roi.csv.xlsx
+++ b/config/acquisitionConfig/roi.csv.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="765" uniqueCount="757">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="773" uniqueCount="765">
   <si>
     <t>Angle</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -2311,6 +2311,30 @@
   </si>
   <si>
     <t>[650 100]</t>
+  </si>
+  <si>
+    <t>NiLattice10MHzGwCavity</t>
+  </si>
+  <si>
+    <t>[]</t>
+  </si>
+  <si>
+    <t>[1 1]</t>
+  </si>
+  <si>
+    <t>[100 100]</t>
+  </si>
+  <si>
+    <t>NiLattice10MHzGwCavity</t>
+  </si>
+  <si>
+    <t>[]</t>
+  </si>
+  <si>
+    <t>[1 1]</t>
+  </si>
+  <si>
+    <t>[100 100]</t>
   </si>
 </sst>
 </file>
@@ -2637,7 +2661,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K43"/>
+  <dimension ref="A1:K44"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="26.5703125" customWidth="true"/>
@@ -4155,6 +4179,41 @@
         <v>756</v>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" s="0" t="s">
+        <v>761</v>
+      </c>
+      <c r="B44" s="0">
+        <v>1050</v>
+      </c>
+      <c r="C44" s="0">
+        <v>1450</v>
+      </c>
+      <c r="D44" s="0">
+        <v>1260</v>
+      </c>
+      <c r="E44" s="0">
+        <v>1350</v>
+      </c>
+      <c r="F44" s="0">
+        <v>2160</v>
+      </c>
+      <c r="G44" s="0">
+        <v>2560</v>
+      </c>
+      <c r="H44" s="0">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="I44" s="0" t="s">
+        <v>762</v>
+      </c>
+      <c r="J44" s="0" t="s">
+        <v>763</v>
+      </c>
+      <c r="K44" s="0" t="s">
+        <v>764</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>